<commit_message>
updates syntax in NormalizedLifeStanceBillingReport.script
</commit_message>
<xml_diff>
--- a/Scripts4Scripps.suite/Resources/July 2026 CoCM Billing Report with Removed Patient PII.xlsx
+++ b/Scripts4Scripps.suite/Resources/July 2026 CoCM Billing Report with Removed Patient PII.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScriptRepositories\Scripps\Scripts4Scripps.suite\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78DEE218-8202-4F80-835F-064EEB3E4E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAB087EF-C6D1-41EB-9878-DC5E602BD94D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1561,7 +1561,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9684133426923432E-2"/>
+        <fgColor theme="0" tint="-4.9623096407971433E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -9660,7 +9660,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B5:S146" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="B5:S146" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="17" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>